<commit_message>
feat(working): add department, position and salary structure entities
- Create new entity classes (Department, Position, PaSalaryScale, PaSalaryGrade, PaSalaryLevel) in separate files
- Add sample data for departments, positions, and salary structures to AppDataContext
- Extend HuWorkingController to include department and position dropdowns in Excel template
- Add data validation and hidden ID columns for department and position selection
- Enhance import logic to parse additional fields (decision number, dates, department, position)
- Remove entity definitions from controller file and organize them properly
</commit_message>
<xml_diff>
--- a/ImportExportExcellApi/Templates/HU_WORKING_BASE.xlsx
+++ b/ImportExportExcellApi/Templates/HU_WORKING_BASE.xlsx
@@ -1388,21 +1388,10 @@
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.1428571428571" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="23.0095238095238" customWidth="1"/>
-    <col min="3" max="4" width="16.1428571428571" customWidth="1"/>
-    <col min="5" max="5" width="16.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="26.7142857142857" customWidth="1"/>
-    <col min="7" max="7" width="19.3238095238095" customWidth="1"/>
-    <col min="8" max="9" width="22.1809523809524" customWidth="1"/>
-    <col min="10" max="10" width="26.7238095238095" customWidth="1"/>
-    <col min="11" max="11" width="17.7142857142857" customWidth="1"/>
+    <col min="2" max="11" width="22.7142857142857" customWidth="1"/>
     <col min="12" max="12" width="23.5333333333333" customWidth="1"/>
-    <col min="13" max="13" width="15.1428571428571" customWidth="1"/>
-    <col min="14" max="14" width="17.5714285714286" customWidth="1"/>
-    <col min="15" max="15" width="16.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="16.2857142857143" customWidth="1"/>
-    <col min="17" max="17" width="15.1428571428571" customWidth="1"/>
-    <col min="18" max="18" width="14.1047619047619" customWidth="1"/>
+    <col min="13" max="13" width="25.7142857142857" customWidth="1"/>
+    <col min="14" max="18" width="22.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:18">

</xml_diff>